<commit_message>
Excel al día: ARG vs EGY en Atlanta, rival de SUI por confirmar y sin empates en las listas
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quiniela Octavos 2026.xlsx
+++ b/Quiniela Octavos 2026.xlsx
@@ -2,22 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiniela" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,36 +25,56 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFD447"/>
-      <sz val="18"/>
+      <color rgb="FFFFD447"/>
+      <sz val="19"/>
     </font>
     <font>
-      <color rgb="00F2F7F4"/>
-      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="19"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFD447"/>
-      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FFF2F7F4"/>
+      <sz val="14"/>
     </font>
     <font>
-      <color rgb="00F2F7F4"/>
-      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="14"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00F2F7F4"/>
-      <sz val="9"/>
+      <color rgb="FFFFD447"/>
+      <sz val="14"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00F2F7F4"/>
-      <sz val="11"/>
+      <color rgb="FFF2F7F4"/>
+      <sz val="14"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <family val="2"/>
       <i val="1"/>
-      <sz val="10"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFD447"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="6">
@@ -67,26 +86,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000B3D2E"/>
+        <fgColor rgb="FF0B3D2E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F4A37"/>
+        <fgColor rgb="FF0F4A37"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00081F16"/>
+        <fgColor rgb="FF081F16"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAF2EE"/>
+        <fgColor rgb="FFEAF2EE"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -96,54 +115,134 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="009FB8AC"/>
+        <color rgb="FF9FB8AC"/>
       </left>
       <right style="thin">
-        <color rgb="009FB8AC"/>
+        <color rgb="FF9FB8AC"/>
       </right>
       <top style="thin">
-        <color rgb="009FB8AC"/>
+        <color rgb="FF9FB8AC"/>
       </top>
       <bottom style="thin">
-        <color rgb="009FB8AC"/>
+        <color rgb="FF9FB8AC"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF9FB8AC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF9FB8AC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF9FB8AC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF9FB8AC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF9FB8AC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF9FB8AC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF9FB8AC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF9FB8AC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF9FB8AC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF9FB8AC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF9FB8AC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF9FB8AC"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -507,26 +606,27 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="24"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="15" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" style="3" min="1" max="1"/>
+    <col width="17" customWidth="1" style="3" min="2" max="2"/>
+    <col width="15" customWidth="1" style="3" min="3" max="3"/>
+    <col width="13" customWidth="1" style="3" min="4" max="4"/>
+    <col width="15" customWidth="1" style="3" min="5" max="5"/>
+    <col width="13" customWidth="1" style="3" min="6" max="6"/>
+    <col width="15" customWidth="1" style="3" min="7" max="7"/>
+    <col width="13" customWidth="1" style="3" min="8" max="8"/>
+    <col width="15" customWidth="1" style="3" min="9" max="9"/>
+    <col width="13" customWidth="1" style="3" min="10" max="10"/>
+    <col width="15" customWidth="1" style="3" min="11" max="11"/>
+    <col width="13" customWidth="1" style="3" min="12" max="12"/>
+    <col width="15" customWidth="1" style="3" min="13" max="13"/>
+    <col width="13" customWidth="1" style="3" min="14" max="14"/>
+    <col width="15" customWidth="1" style="3" min="15" max="15"/>
+    <col width="13" customWidth="1" style="3" min="16" max="16"/>
+    <col width="15" customWidth="1" style="3" min="17" max="17"/>
+    <col width="13" customWidth="1" style="3" min="18" max="18"/>
+    <col width="8.88671875" customWidth="1" style="3" min="19" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -536,490 +636,510 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="46" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>REGLAS: 1 punto por atinarle al ganador (o al empate) · 3 puntos por el marcador exacto (el empate también cuenta: 0-0, 1-1…) · 5 puntos si tu FAVORITO gana el Mundial · Todo se califica a los 90 minutos, los penales NO cuentan · Apuesta: $1,000 por jugador · ENTREGA ANTES DEL SÁBADO 4 DE JULIO, 9:00 AM</t>
+    <row r="2" ht="46.05" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>REGLAS: 1 punto por atinarle al ganador · 3 puntos por el marcador exacto · 5 puntos si tu FAVORITO gana el Mundial · No hay empates: siempre gana alguien; si hay penales, cuenta el marcador final de los penales · Apuesta: $1,000 por jugador · ENTREGA ANTES DEL SÁBADO 4 DE JULIO, 9:00 AM</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>JUGADOR</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>🏆 FAVORITO
 (campeón del Mundial)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Canadá vs Marruecos</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Paraguay vs Francia</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="15" t="inlineStr">
         <is>
           <t>México vs Inglaterra</t>
         </is>
       </c>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="15" t="inlineStr">
         <is>
           <t>Brasil vs Noruega</t>
         </is>
       </c>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="J4" s="16" t="n"/>
+      <c r="K4" s="15" t="inlineStr">
         <is>
           <t>Portugal vs España</t>
         </is>
       </c>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Estados Unidos vs Bélgica</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>Por definir</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="n"/>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="L4" s="16" t="n"/>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>USA vs Bélgica</t>
+        </is>
+      </c>
+      <c r="N4" s="16" t="n"/>
+      <c r="O4" s="15" t="inlineStr">
+        <is>
+          <t>Argentina vs Egipto</t>
+        </is>
+      </c>
+      <c r="P4" s="16" t="n"/>
+      <c r="Q4" s="15" t="inlineStr">
         <is>
           <t>Suiza vs Por definir</t>
         </is>
       </c>
-      <c r="R4" s="3" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="R4" s="16" t="n"/>
+    </row>
+    <row r="5" ht="63.6" customHeight="1">
+      <c r="A5" s="17" t="n"/>
+      <c r="B5" s="17" t="n"/>
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Sáb 4 jul · Houston</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Sáb 4 jul · Filadelfia</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Dom 5 jul 18:00 · Azteca</t>
         </is>
       </c>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>Dom 5 jul 14:00 · NY</t>
         </is>
       </c>
-      <c r="J5" s="4" t="n"/>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="J5" s="16" t="n"/>
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>Lun 6 jul 13:00 · Dallas</t>
         </is>
       </c>
-      <c r="L5" s="4" t="n"/>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="L5" s="16" t="n"/>
+      <c r="M5" s="7" t="inlineStr">
         <is>
           <t>Lun 6 jul · Seattle</t>
         </is>
       </c>
-      <c r="N5" s="4" t="n"/>
-      <c r="O5" s="4" t="inlineStr">
-        <is>
-          <t>6–7 jul · ARG/CabVerde vs AUS/Egipto</t>
-        </is>
-      </c>
-      <c r="P5" s="4" t="n"/>
-      <c r="Q5" s="4" t="inlineStr">
-        <is>
-          <t>Mar 7 jul · Vancouver (rival: COL/Ghana)</t>
-        </is>
-      </c>
-      <c r="R5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="N5" s="16" t="n"/>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
+          <t>Mar 7 jul · Atlanta</t>
+        </is>
+      </c>
+      <c r="P5" s="16" t="n"/>
+      <c r="Q5" s="7" t="inlineStr">
+        <is>
+          <t>Mar 7 jul · Vancouver (rival: COL/Ghana, por confirmar)</t>
+        </is>
+      </c>
+      <c r="R5" s="16" t="n"/>
+    </row>
+    <row r="6" ht="34.8" customHeight="1">
+      <c r="A6" s="18" t="n"/>
+      <c r="B6" s="18" t="n"/>
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>¿Quién gana?</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Marcador (ej. 2-1)</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>¿Quién gana?</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Marcador (ej. 2-1)</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>¿Quién gana?</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>Marcador (ej. 2-1)</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>¿Quién gana?</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="9" t="inlineStr">
         <is>
           <t>Marcador (ej. 2-1)</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>¿Quién gana?</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="L6" s="9" t="inlineStr">
         <is>
           <t>Marcador (ej. 2-1)</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="M6" s="9" t="inlineStr">
         <is>
           <t>¿Quién gana?</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="N6" s="9" t="inlineStr">
         <is>
           <t>Marcador (ej. 2-1)</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="O6" s="9" t="inlineStr">
         <is>
           <t>¿Quién gana?</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr">
+      <c r="P6" s="9" t="inlineStr">
         <is>
           <t>Marcador (ej. 2-1)</t>
         </is>
       </c>
-      <c r="Q6" s="5" t="inlineStr">
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>¿Quién gana?</t>
         </is>
       </c>
-      <c r="R6" s="5" t="inlineStr">
+      <c r="R6" s="9" t="inlineStr">
         <is>
           <t>Marcador (ej. 2-1)</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="7" ht="22.05" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Imelda</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
-      <c r="O7" s="7" t="n"/>
-      <c r="P7" s="7" t="n"/>
-      <c r="Q7" s="7" t="n"/>
-      <c r="R7" s="7" t="n"/>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="11" t="n"/>
+      <c r="I7" s="11" t="n"/>
+      <c r="J7" s="11" t="n"/>
+      <c r="K7" s="11" t="n"/>
+      <c r="L7" s="11" t="n"/>
+      <c r="M7" s="11" t="n"/>
+      <c r="N7" s="11" t="n"/>
+      <c r="O7" s="11" t="n"/>
+      <c r="P7" s="11" t="n"/>
+      <c r="Q7" s="11" t="n"/>
+      <c r="R7" s="11" t="n"/>
+    </row>
+    <row r="8" ht="22.05" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Franca</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="8" t="n"/>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="8" t="n"/>
-      <c r="I8" s="8" t="n"/>
-      <c r="J8" s="8" t="n"/>
-      <c r="K8" s="8" t="n"/>
-      <c r="L8" s="8" t="n"/>
-      <c r="M8" s="8" t="n"/>
-      <c r="N8" s="8" t="n"/>
-      <c r="O8" s="8" t="n"/>
-      <c r="P8" s="8" t="n"/>
-      <c r="Q8" s="8" t="n"/>
-      <c r="R8" s="8" t="n"/>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="12" t="n"/>
+      <c r="L8" s="12" t="n"/>
+      <c r="M8" s="12" t="n"/>
+      <c r="N8" s="12" t="n"/>
+      <c r="O8" s="12" t="n"/>
+      <c r="P8" s="12" t="n"/>
+      <c r="Q8" s="12" t="n"/>
+      <c r="R8" s="12" t="n"/>
+    </row>
+    <row r="9" ht="22.05" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Paola</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
-      <c r="O9" s="7" t="n"/>
-      <c r="P9" s="7" t="n"/>
-      <c r="Q9" s="7" t="n"/>
-      <c r="R9" s="7" t="n"/>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="11" t="n"/>
+      <c r="I9" s="11" t="n"/>
+      <c r="J9" s="11" t="n"/>
+      <c r="K9" s="11" t="n"/>
+      <c r="L9" s="11" t="n"/>
+      <c r="M9" s="11" t="n"/>
+      <c r="N9" s="11" t="n"/>
+      <c r="O9" s="11" t="n"/>
+      <c r="P9" s="11" t="n"/>
+      <c r="Q9" s="11" t="n"/>
+      <c r="R9" s="11" t="n"/>
+    </row>
+    <row r="10" ht="22.05" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Caroline</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n"/>
-      <c r="C10" s="8" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="8" t="n"/>
-      <c r="I10" s="8" t="n"/>
-      <c r="J10" s="8" t="n"/>
-      <c r="K10" s="8" t="n"/>
-      <c r="L10" s="8" t="n"/>
-      <c r="M10" s="8" t="n"/>
-      <c r="N10" s="8" t="n"/>
-      <c r="O10" s="8" t="n"/>
-      <c r="P10" s="8" t="n"/>
-      <c r="Q10" s="8" t="n"/>
-      <c r="R10" s="8" t="n"/>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="12" t="n"/>
+      <c r="E10" s="12" t="n"/>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="12" t="n"/>
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="12" t="n"/>
+      <c r="L10" s="12" t="n"/>
+      <c r="M10" s="12" t="n"/>
+      <c r="N10" s="12" t="n"/>
+      <c r="O10" s="12" t="n"/>
+      <c r="P10" s="12" t="n"/>
+      <c r="Q10" s="12" t="n"/>
+      <c r="R10" s="12" t="n"/>
+    </row>
+    <row r="11" ht="22.05" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Daniel</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7" t="n"/>
-      <c r="N11" s="7" t="n"/>
-      <c r="O11" s="7" t="n"/>
-      <c r="P11" s="7" t="n"/>
-      <c r="Q11" s="7" t="n"/>
-      <c r="R11" s="7" t="n"/>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="11" t="n"/>
+      <c r="I11" s="11" t="n"/>
+      <c r="J11" s="11" t="n"/>
+      <c r="K11" s="11" t="n"/>
+      <c r="L11" s="11" t="n"/>
+      <c r="M11" s="11" t="n"/>
+      <c r="N11" s="11" t="n"/>
+      <c r="O11" s="11" t="n"/>
+      <c r="P11" s="11" t="n"/>
+      <c r="Q11" s="11" t="n"/>
+      <c r="R11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="22.05" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Angie</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="8" t="n"/>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="8" t="n"/>
-      <c r="G12" s="8" t="n"/>
-      <c r="H12" s="8" t="n"/>
-      <c r="I12" s="8" t="n"/>
-      <c r="J12" s="8" t="n"/>
-      <c r="K12" s="8" t="n"/>
-      <c r="L12" s="8" t="n"/>
-      <c r="M12" s="8" t="n"/>
-      <c r="N12" s="8" t="n"/>
-      <c r="O12" s="8" t="n"/>
-      <c r="P12" s="8" t="n"/>
-      <c r="Q12" s="8" t="n"/>
-      <c r="R12" s="8" t="n"/>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="12" t="n"/>
+      <c r="H12" s="12" t="n"/>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="12" t="n"/>
+      <c r="L12" s="12" t="n"/>
+      <c r="M12" s="12" t="n"/>
+      <c r="N12" s="12" t="n"/>
+      <c r="O12" s="12" t="n"/>
+      <c r="P12" s="12" t="n"/>
+      <c r="Q12" s="12" t="n"/>
+      <c r="R12" s="12" t="n"/>
+    </row>
+    <row r="13" ht="22.05" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Estela</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="7" t="n"/>
-      <c r="I13" s="7" t="n"/>
-      <c r="J13" s="7" t="n"/>
-      <c r="K13" s="7" t="n"/>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7" t="n"/>
-      <c r="N13" s="7" t="n"/>
-      <c r="O13" s="7" t="n"/>
-      <c r="P13" s="7" t="n"/>
-      <c r="Q13" s="7" t="n"/>
-      <c r="R13" s="7" t="n"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="11" t="n"/>
+      <c r="I13" s="11" t="n"/>
+      <c r="J13" s="11" t="n"/>
+      <c r="K13" s="11" t="n"/>
+      <c r="L13" s="11" t="n"/>
+      <c r="M13" s="11" t="n"/>
+      <c r="N13" s="11" t="n"/>
+      <c r="O13" s="11" t="n"/>
+      <c r="P13" s="11" t="n"/>
+      <c r="Q13" s="11" t="n"/>
+      <c r="R13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="22.05" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>David</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="8" t="n"/>
-      <c r="G14" s="8" t="n"/>
-      <c r="H14" s="8" t="n"/>
-      <c r="I14" s="8" t="n"/>
-      <c r="J14" s="8" t="n"/>
-      <c r="K14" s="8" t="n"/>
-      <c r="L14" s="8" t="n"/>
-      <c r="M14" s="8" t="n"/>
-      <c r="N14" s="8" t="n"/>
-      <c r="O14" s="8" t="n"/>
-      <c r="P14" s="8" t="n"/>
-      <c r="Q14" s="8" t="n"/>
-      <c r="R14" s="8" t="n"/>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="12" t="n"/>
+      <c r="H14" s="12" t="n"/>
+      <c r="I14" s="12" t="n"/>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="12" t="n"/>
+      <c r="L14" s="12" t="n"/>
+      <c r="M14" s="12" t="n"/>
+      <c r="N14" s="12" t="n"/>
+      <c r="O14" s="12" t="n"/>
+      <c r="P14" s="12" t="n"/>
+      <c r="Q14" s="12" t="n"/>
+      <c r="R14" s="12" t="n"/>
+    </row>
+    <row r="15" ht="22.05" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Alexa</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
-      <c r="G15" s="7" t="n"/>
-      <c r="H15" s="7" t="n"/>
-      <c r="I15" s="7" t="n"/>
-      <c r="J15" s="7" t="n"/>
-      <c r="K15" s="7" t="n"/>
-      <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7" t="n"/>
-      <c r="N15" s="7" t="n"/>
-      <c r="O15" s="7" t="n"/>
-      <c r="P15" s="7" t="n"/>
-      <c r="Q15" s="7" t="n"/>
-      <c r="R15" s="7" t="n"/>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="6" t="inlineStr"/>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="8" t="n"/>
-      <c r="G16" s="8" t="n"/>
-      <c r="H16" s="8" t="n"/>
-      <c r="I16" s="8" t="n"/>
-      <c r="J16" s="8" t="n"/>
-      <c r="K16" s="8" t="n"/>
-      <c r="L16" s="8" t="n"/>
-      <c r="M16" s="8" t="n"/>
-      <c r="N16" s="8" t="n"/>
-      <c r="O16" s="8" t="n"/>
-      <c r="P16" s="8" t="n"/>
-      <c r="Q16" s="8" t="n"/>
-      <c r="R16" s="8" t="n"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="6" t="inlineStr"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="7" t="n"/>
-      <c r="I17" s="7" t="n"/>
-      <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="n"/>
-      <c r="M17" s="7" t="n"/>
-      <c r="N17" s="7" t="n"/>
-      <c r="O17" s="7" t="n"/>
-      <c r="P17" s="7" t="n"/>
-      <c r="Q17" s="7" t="n"/>
-      <c r="R17" s="7" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="6" t="inlineStr"/>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="8" t="n"/>
-      <c r="E18" s="8" t="n"/>
-      <c r="F18" s="8" t="n"/>
-      <c r="G18" s="8" t="n"/>
-      <c r="H18" s="8" t="n"/>
-      <c r="I18" s="8" t="n"/>
-      <c r="J18" s="8" t="n"/>
-      <c r="K18" s="8" t="n"/>
-      <c r="L18" s="8" t="n"/>
-      <c r="M18" s="8" t="n"/>
-      <c r="N18" s="8" t="n"/>
-      <c r="O18" s="8" t="n"/>
-      <c r="P18" s="8" t="n"/>
-      <c r="Q18" s="8" t="n"/>
-      <c r="R18" s="8" t="n"/>
-    </row>
-    <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>CÓMO LLENAR: en '¿Quién gana?' elige de la lista (equipo o EMPATE). En 'Marcador' escribe los goles, ej. 2-1 (si crees empate: 0-0, 1-1…). Elige tu FAVORITO para campeón. En los cruces por definir, elige al equipo que creas que estará ahí y ganará.</t>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
+      <c r="H15" s="11" t="n"/>
+      <c r="I15" s="11" t="n"/>
+      <c r="J15" s="11" t="n"/>
+      <c r="K15" s="11" t="n"/>
+      <c r="L15" s="11" t="n"/>
+      <c r="M15" s="11" t="n"/>
+      <c r="N15" s="11" t="n"/>
+      <c r="O15" s="11" t="n"/>
+      <c r="P15" s="11" t="n"/>
+      <c r="Q15" s="11" t="n"/>
+      <c r="R15" s="11" t="n"/>
+    </row>
+    <row r="16" ht="22.05" customHeight="1">
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="12" t="n"/>
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="12" t="n"/>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="12" t="n"/>
+      <c r="G16" s="12" t="n"/>
+      <c r="H16" s="12" t="n"/>
+      <c r="I16" s="12" t="n"/>
+      <c r="J16" s="12" t="n"/>
+      <c r="K16" s="12" t="n"/>
+      <c r="L16" s="12" t="n"/>
+      <c r="M16" s="12" t="n"/>
+      <c r="N16" s="12" t="n"/>
+      <c r="O16" s="12" t="n"/>
+      <c r="P16" s="12" t="n"/>
+      <c r="Q16" s="12" t="n"/>
+      <c r="R16" s="12" t="n"/>
+    </row>
+    <row r="17" ht="22.05" customHeight="1">
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="11" t="n"/>
+      <c r="I17" s="11" t="n"/>
+      <c r="J17" s="11" t="n"/>
+      <c r="K17" s="11" t="n"/>
+      <c r="L17" s="11" t="n"/>
+      <c r="M17" s="11" t="n"/>
+      <c r="N17" s="11" t="n"/>
+      <c r="O17" s="11" t="n"/>
+      <c r="P17" s="11" t="n"/>
+      <c r="Q17" s="11" t="n"/>
+      <c r="R17" s="11" t="n"/>
+    </row>
+    <row r="18" ht="22.05" customHeight="1">
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="12" t="n"/>
+      <c r="H18" s="12" t="n"/>
+      <c r="I18" s="12" t="n"/>
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="12" t="n"/>
+      <c r="L18" s="12" t="n"/>
+      <c r="M18" s="12" t="n"/>
+      <c r="N18" s="12" t="n"/>
+      <c r="O18" s="12" t="n"/>
+      <c r="P18" s="12" t="n"/>
+      <c r="Q18" s="12" t="n"/>
+      <c r="R18" s="12" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="n"/>
+      <c r="K19" s="13" t="n"/>
+      <c r="L19" s="13" t="n"/>
+      <c r="M19" s="13" t="n"/>
+      <c r="N19" s="13" t="n"/>
+      <c r="O19" s="13" t="n"/>
+      <c r="P19" s="13" t="n"/>
+      <c r="Q19" s="13" t="n"/>
+      <c r="R19" s="13" t="n"/>
+    </row>
+    <row r="20" ht="40.05" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>CÓMO LLENAR: en '¿Quién gana?' elige al equipo (no hay empates: si hay penales, cuenta el marcador final de los penales). En 'Marcador' escribe los goles, ej. 2-1. Elige tu FAVORITO para campeón. En el cruce por definir, elige al equipo que creas que estará ahí y ganará.</t>
         </is>
       </c>
     </row>
@@ -1049,33 +1169,34 @@
   </mergeCells>
   <dataValidations count="9">
     <dataValidation sqref="B7:B18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"México,Inglaterra,Brasil,Noruega,Paraguay,Francia,Canadá,Marruecos,Portugal,España,Estados Unidos,Bélgica,Suiza,Argentina,Cabo Verde,Australia,Egipto,Colombia,Ghana"</formula1>
+      <formula1>"México,Inglaterra,Brasil,Noruega,Paraguay,Francia,Canadá,Marruecos,Portugal,España,Estados Unidos,Bélgica,Suiza,Argentina,Egipto,Colombia,Ghana"</formula1>
     </dataValidation>
     <dataValidation sqref="C7:C18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Canadá,EMPATE,Marruecos"</formula1>
+      <formula1>"Canadá,Marruecos"</formula1>
     </dataValidation>
     <dataValidation sqref="E7:E18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Paraguay,EMPATE,Francia"</formula1>
+      <formula1>"Paraguay,Francia"</formula1>
     </dataValidation>
     <dataValidation sqref="G7:G18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"México,EMPATE,Inglaterra"</formula1>
+      <formula1>"México,Inglaterra"</formula1>
     </dataValidation>
     <dataValidation sqref="I7:I18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Brasil,EMPATE,Noruega"</formula1>
+      <formula1>"Brasil,Noruega"</formula1>
     </dataValidation>
     <dataValidation sqref="K7:K18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Portugal,EMPATE,España"</formula1>
+      <formula1>"Portugal,España"</formula1>
     </dataValidation>
     <dataValidation sqref="M7:M18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Estados Unidos,EMPATE,Bélgica"</formula1>
+      <formula1>"Estados Unidos,Bélgica"</formula1>
     </dataValidation>
     <dataValidation sqref="O7:O18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Argentina,Cabo Verde,EMPATE,Australia,Egipto"</formula1>
+      <formula1>"Argentina,Egipto"</formula1>
     </dataValidation>
     <dataValidation sqref="Q7:Q18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Suiza,EMPATE,Colombia,Ghana"</formula1>
+      <formula1>"Suiza,Colombia,Ghana"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" scale="47"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARG-CPV sigue en juego: el rival de EGY vuelve a 'por definir'; reglas alineadas a la izquierda y encabezado 'Mundial 2026 · Attrapi'
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quiniela Octavos 2026.xlsx
+++ b/Quiniela Octavos 2026.xlsx
@@ -693,7 +693,7 @@
       <c r="N4" s="16" t="n"/>
       <c r="O4" s="15" t="inlineStr">
         <is>
-          <t>Argentina vs Egipto</t>
+          <t>ARG/CabVerde vs Egipto</t>
         </is>
       </c>
       <c r="P4" s="16" t="n"/>
@@ -745,7 +745,7 @@
       <c r="N5" s="16" t="n"/>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>Mar 7 jul · Atlanta</t>
+          <t>Mar 7 jul · Atlanta (Egipto ya clasificó; falta ARG vs CPV)</t>
         </is>
       </c>
       <c r="P5" s="16" t="n"/>
@@ -1169,7 +1169,7 @@
   </mergeCells>
   <dataValidations count="9">
     <dataValidation sqref="B7:B18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"México,Inglaterra,Brasil,Noruega,Paraguay,Francia,Canadá,Marruecos,Portugal,España,Estados Unidos,Bélgica,Suiza,Argentina,Egipto,Colombia,Ghana"</formula1>
+      <formula1>"México,Inglaterra,Brasil,Noruega,Paraguay,Francia,Canadá,Marruecos,Portugal,España,Estados Unidos,Bélgica,Suiza,Argentina,Cabo Verde,Egipto,Colombia,Ghana"</formula1>
     </dataValidation>
     <dataValidation sqref="C7:C18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
       <formula1>"Canadá,Marruecos"</formula1>
@@ -1190,7 +1190,7 @@
       <formula1>"Estados Unidos,Bélgica"</formula1>
     </dataValidation>
     <dataValidation sqref="O7:O18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Argentina,Egipto"</formula1>
+      <formula1>"Argentina,Cabo Verde,Egipto"</formula1>
     </dataValidation>
     <dataValidation sqref="Q7:Q18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
       <formula1>"Suiza,Colombia,Ghana"</formula1>

</xml_diff>

<commit_message>
Argentina venció 3-2 a Cabo Verde en tiempo extra: octavos ARG vs EGY confirmado en página y Excel
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quiniela Octavos 2026.xlsx
+++ b/Quiniela Octavos 2026.xlsx
@@ -693,7 +693,7 @@
       <c r="N4" s="16" t="n"/>
       <c r="O4" s="15" t="inlineStr">
         <is>
-          <t>ARG/CabVerde vs Egipto</t>
+          <t>Argentina vs Egipto</t>
         </is>
       </c>
       <c r="P4" s="16" t="n"/>
@@ -745,7 +745,7 @@
       <c r="N5" s="16" t="n"/>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>Mar 7 jul · Atlanta (Egipto ya clasificó; falta ARG vs CPV)</t>
+          <t>Mar 7 jul · Atlanta</t>
         </is>
       </c>
       <c r="P5" s="16" t="n"/>
@@ -1169,7 +1169,7 @@
   </mergeCells>
   <dataValidations count="9">
     <dataValidation sqref="B7:B18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"México,Inglaterra,Brasil,Noruega,Paraguay,Francia,Canadá,Marruecos,Portugal,España,Estados Unidos,Bélgica,Suiza,Argentina,Cabo Verde,Egipto,Colombia,Ghana"</formula1>
+      <formula1>"México,Inglaterra,Brasil,Noruega,Paraguay,Francia,Canadá,Marruecos,Portugal,España,Estados Unidos,Bélgica,Suiza,Argentina,Egipto,Colombia,Ghana"</formula1>
     </dataValidation>
     <dataValidation sqref="C7:C18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
       <formula1>"Canadá,Marruecos"</formula1>
@@ -1190,7 +1190,7 @@
       <formula1>"Estados Unidos,Bélgica"</formula1>
     </dataValidation>
     <dataValidation sqref="O7:O18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Argentina,Cabo Verde,Egipto"</formula1>
+      <formula1>"Argentina,Egipto"</formula1>
     </dataValidation>
     <dataValidation sqref="Q7:Q18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
       <formula1>"Suiza,Colombia,Ghana"</formula1>

</xml_diff>

<commit_message>
Excel: vuelve EMPATE a las listas y reglas de 1 o 3 puntos
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quiniela Octavos 2026.xlsx
+++ b/Quiniela Octavos 2026.xlsx
@@ -639,7 +639,7 @@
     <row r="2" ht="46.05" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>REGLAS: 1 punto por atinarle al ganador · 3 puntos por el marcador exacto · 5 puntos si tu FAVORITO gana el Mundial · No hay empates: siempre gana alguien; si hay penales, cuenta el marcador final de los penales · Apuesta: $1,000 por jugador · ENTREGA ANTES DEL SÁBADO 4 DE JULIO, 9:00 AM</t>
+          <t>REGLAS: 1 punto por atinarle al resultado (ganador o EMPATE) · 3 puntos por el marcador exacto · En cada partido ganas 1 o 3 puntos, no se suman · 5 puntos si tu FAVORITO gana el Mundial · Apuesta: $1,000 por jugador · ENTREGA ANTES DEL SÁBADO 4 DE JULIO, 9:00 AM</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
     <row r="20" ht="40.05" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>CÓMO LLENAR: en '¿Quién gana?' elige al equipo (no hay empates: si hay penales, cuenta el marcador final de los penales). En 'Marcador' escribe los goles, ej. 2-1. Elige tu FAVORITO para campeón. En el cruce por definir, elige al equipo que creas que estará ahí y ganará.</t>
+          <t>CÓMO LLENAR: en '¿Quién gana?' elige de la lista (equipo o EMPATE). En 'Marcador' escribe los goles, ej. 2-1 (si crees empate: 0-0, 1-1…). Elige tu FAVORITO para campeón. En el cruce por definir, elige al equipo que creas que estará ahí y ganará.</t>
         </is>
       </c>
     </row>
@@ -1172,28 +1172,28 @@
       <formula1>"México,Inglaterra,Brasil,Noruega,Paraguay,Francia,Canadá,Marruecos,Portugal,España,Estados Unidos,Bélgica,Suiza,Argentina,Egipto,Colombia,Ghana"</formula1>
     </dataValidation>
     <dataValidation sqref="C7:C18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Canadá,Marruecos"</formula1>
+      <formula1>"Canadá,EMPATE,Marruecos"</formula1>
     </dataValidation>
     <dataValidation sqref="E7:E18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Paraguay,Francia"</formula1>
+      <formula1>"Paraguay,EMPATE,Francia"</formula1>
     </dataValidation>
     <dataValidation sqref="G7:G18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"México,Inglaterra"</formula1>
+      <formula1>"México,EMPATE,Inglaterra"</formula1>
     </dataValidation>
     <dataValidation sqref="I7:I18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Brasil,Noruega"</formula1>
+      <formula1>"Brasil,EMPATE,Noruega"</formula1>
     </dataValidation>
     <dataValidation sqref="K7:K18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Portugal,España"</formula1>
+      <formula1>"Portugal,EMPATE,España"</formula1>
     </dataValidation>
     <dataValidation sqref="M7:M18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Estados Unidos,Bélgica"</formula1>
+      <formula1>"Estados Unidos,EMPATE,Bélgica"</formula1>
     </dataValidation>
     <dataValidation sqref="O7:O18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Argentina,Egipto"</formula1>
+      <formula1>"Argentina,EMPATE,Egipto"</formula1>
     </dataValidation>
     <dataValidation sqref="Q7:Q18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Suiza,Colombia,Ghana"</formula1>
+      <formula1>"Suiza,EMPATE,Colombia,Ghana"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Colombia venció 1-0 a Ghana y cierra los octavos: SUI vs COL en Vancouver; pick de penales con +1 punto cuando eliges EMP
- Los 8 cruces de octavos quedan completos en página y Excel
- Al elegir EMP aparece el selector 🥅 para atinarle al ganador de penales (+1 punto)
- Ghana sale de las listas del Excel

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quiniela Octavos 2026.xlsx
+++ b/Quiniela Octavos 2026.xlsx
@@ -699,7 +699,7 @@
       <c r="P4" s="16" t="n"/>
       <c r="Q4" s="15" t="inlineStr">
         <is>
-          <t>Suiza vs Por definir</t>
+          <t>Suiza vs Colombia</t>
         </is>
       </c>
       <c r="R4" s="16" t="n"/>
@@ -751,7 +751,7 @@
       <c r="P5" s="16" t="n"/>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>Mar 7 jul · Vancouver (rival: COL/Ghana, por confirmar)</t>
+          <t>Mar 7 jul · Vancouver</t>
         </is>
       </c>
       <c r="R5" s="16" t="n"/>
@@ -1169,7 +1169,7 @@
   </mergeCells>
   <dataValidations count="9">
     <dataValidation sqref="B7:B18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"México,Inglaterra,Brasil,Noruega,Paraguay,Francia,Canadá,Marruecos,Portugal,España,Estados Unidos,Bélgica,Suiza,Argentina,Egipto,Colombia,Ghana"</formula1>
+      <formula1>"México,Inglaterra,Brasil,Noruega,Paraguay,Francia,Canadá,Marruecos,Portugal,España,Estados Unidos,Bélgica,Suiza,Argentina,Egipto,Colombia"</formula1>
     </dataValidation>
     <dataValidation sqref="C7:C18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
       <formula1>"Canadá,EMPATE,Marruecos"</formula1>
@@ -1193,7 +1193,7 @@
       <formula1>"Argentina,EMPATE,Egipto"</formula1>
     </dataValidation>
     <dataValidation sqref="Q7:Q18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Opción inválida" error="Elige una opción de la lista." type="list">
-      <formula1>"Suiza,EMPATE,Colombia,Ghana"</formula1>
+      <formula1>"Suiza,EMPATE,Colombia"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>